<commit_message>
Updated Mentor Mentee upload status
</commit_message>
<xml_diff>
--- a/server/data/MENTOR-MENTEE.xlsx
+++ b/server/data/MENTOR-MENTEE.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
   <si>
     <t>mentor_rollno</t>
   </si>
@@ -26,6 +26,27 @@
   </si>
   <si>
     <t>date</t>
+  </si>
+  <si>
+    <t>STU001</t>
+  </si>
+  <si>
+    <t>7376242AD136</t>
+  </si>
+  <si>
+    <t>c programming</t>
+  </si>
+  <si>
+    <t>18-08-2025</t>
+  </si>
+  <si>
+    <t>STU002</t>
+  </si>
+  <si>
+    <t>7376242AD336</t>
+  </si>
+  <si>
+    <t>Pyhton</t>
   </si>
 </sst>
 </file>
@@ -296,6 +317,40 @@
         <v>4</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>